<commit_message>
Sběr 2026-09-21: 2 přijato
</commit_message>
<xml_diff>
--- a/data/kola/2026-09-21/vysledky.xlsx
+++ b/data/kola/2026-09-21/vysledky.xlsx
@@ -556,9 +556,9 @@
           <t>petr test</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>chybí</t>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>odevzdal</t>
         </is>
       </c>
     </row>
@@ -636,8 +636,8 @@
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="21.5" customWidth="1" min="5" max="5"/>
     <col width="21.5" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
@@ -724,16 +724,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="13" t="n">
-        <v>46286.76923611111</v>
+        <v>46286.7746875</v>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>petr@42prague.com</t>
+          <t>peta.simcak@gmail.com</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>petr prace</t>
+          <t>Peta Simcak</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr"/>
@@ -746,17 +746,30 @@
       <c r="L4" s="14" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="B5" s="15" t="n"/>
-      <c r="C5" s="15" t="n"/>
-      <c r="D5" s="15" t="n"/>
-      <c r="E5" s="15" t="n"/>
-      <c r="F5" s="15" t="n"/>
-      <c r="G5" s="15" t="n"/>
-      <c r="H5" s="15" t="n"/>
-      <c r="I5" s="15" t="n"/>
-      <c r="J5" s="15" t="n"/>
-      <c r="K5" s="15" t="n"/>
-      <c r="L5" s="15" t="n"/>
+      <c r="A5" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>46286.76923611111</v>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>petr@42prague.com</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>petr prace</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr"/>
+      <c r="F5" s="14" t="inlineStr"/>
+      <c r="G5" s="14" t="inlineStr"/>
+      <c r="H5" s="14" t="inlineStr"/>
+      <c r="I5" s="14" t="inlineStr"/>
+      <c r="J5" s="14" t="inlineStr"/>
+      <c r="K5" s="14" t="inlineStr"/>
+      <c r="L5" s="14" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="B6" s="15" t="n"/>
@@ -800,7 +813,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Kolo 2026-09-21 · lístků v bloku 1 z 5 · hodnocení jsou zapsána bez mezer (++ nikoli + +), jak je čte matice.</t>
+          <t>Kolo 2026-09-21 · lístků v bloku 2 z 5 · hodnocení jsou zapsána bez mezer (++ nikoli + +), jak je čte matice.</t>
         </is>
       </c>
     </row>

</xml_diff>